<commit_message>
cambios en tablas latex
</commit_message>
<xml_diff>
--- a/resultados/resultados_RS_cv_vs_test.xlsx
+++ b/resultados/resultados_RS_cv_vs_test.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3362,7 +3362,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>20</v>
       </c>
@@ -3415,7 +3415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -3468,7 +3468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>23</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>23</v>
       </c>
@@ -3916,7 +3916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
@@ -3967,7 +3967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>19</v>
       </c>
@@ -4022,7 +4022,7 @@
   <autoFilter ref="A1:S13">
     <filterColumn colId="8">
       <filters>
-        <filter val="0"/>
+        <filter val="1"/>
       </filters>
     </filterColumn>
     <sortState ref="A4:S12">

</xml_diff>